<commit_message>
Enable Curo maps and trip planning
Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/abha-places-data.xlsx
+++ b/abha-places-data.xlsx
@@ -884,11 +884,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A3257BD-E724-4F19-BA1F-341C9C946AC8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{9A3257BD-E724-4F19-BA1F-341C9C946AC8}">
   <dimension ref="A1:M21"/>
-  <sheetFormatPr defaultColWidth="25.9140625" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="25.9140625" defaultRowHeight="14" ns3:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ns3:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -929,7 +929,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ns3:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -970,7 +970,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" ns3:dyDescent="0.3">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -1011,7 +1011,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ns3:dyDescent="0.3">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -1052,7 +1052,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" ns3:dyDescent="0.3">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -1093,7 +1093,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" ns3:dyDescent="0.3">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -1134,7 +1134,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" ns3:dyDescent="0.3">
       <c r="A7" t="s">
         <v>48</v>
       </c>
@@ -1175,7 +1175,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ns3:dyDescent="0.3">
       <c r="A8" t="s">
         <v>56</v>
       </c>
@@ -1216,7 +1216,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" ns3:dyDescent="0.3">
       <c r="A9" t="s">
         <v>64</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" ns3:dyDescent="0.3">
       <c r="A10" t="s">
         <v>71</v>
       </c>
@@ -1298,7 +1298,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" ns3:dyDescent="0.3">
       <c r="A11" t="s">
         <v>79</v>
       </c>
@@ -1339,7 +1339,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" ns3:dyDescent="0.3">
       <c r="A12" t="s">
         <v>87</v>
       </c>
@@ -1380,7 +1380,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" ns3:dyDescent="0.3">
       <c r="A13" t="s">
         <v>97</v>
       </c>
@@ -1421,7 +1421,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" ns3:dyDescent="0.3">
       <c r="A14" t="s">
         <v>102</v>
       </c>
@@ -1462,7 +1462,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" ns3:dyDescent="0.3">
       <c r="A15" t="s">
         <v>109</v>
       </c>
@@ -1503,7 +1503,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" ns3:dyDescent="0.3">
       <c r="A16" t="s">
         <v>117</v>
       </c>
@@ -1516,6 +1516,11 @@
       <c r="D16" t="s">
         <v>120</v>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/LbSaGp1SnfYA1xJo7?g_st=iw</t>
+        </is>
+      </c>
       <c r="F16" t="s">
         <v>121</v>
       </c>
@@ -1541,7 +1546,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" ns3:dyDescent="0.3">
       <c r="A17" t="s">
         <v>123</v>
       </c>
@@ -1582,39 +1587,39 @@
         <v>151</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" ns3:dyDescent="0.3">
       <c r="D18" s="2"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" ns3:dyDescent="0.3">
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" ns3:dyDescent="0.3">
       <c r="D20" s="2"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" ns3:dyDescent="0.3">
       <c r="J21" t="s">
         <v>152</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{97722929-2038-4234-80FD-4DEF83C3C193}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{9D411408-40F9-4801-AE8C-3AEE32AB4F6F}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{AA8D31E7-236A-4B13-848B-9E3CB9E37B43}"/>
-    <hyperlink ref="E5" r:id="rId4" xr:uid="{55A960DF-E1FD-4872-B20A-AE949F89215A}"/>
-    <hyperlink ref="E6" r:id="rId5" xr:uid="{413665A7-BF97-4CEE-8C6E-ECC7C0E43443}"/>
-    <hyperlink ref="E7" r:id="rId6" xr:uid="{827A3105-6114-485F-A80C-88929EA91C3A}"/>
-    <hyperlink ref="E8" r:id="rId7" xr:uid="{CDB97694-3BF6-4F69-B0C0-E925ADBCD30B}"/>
-    <hyperlink ref="E9" r:id="rId8" xr:uid="{FDF973CA-B570-43F4-9F76-88BAF56A975E}"/>
-    <hyperlink ref="E10" r:id="rId9" xr:uid="{B7BB62B8-3423-4809-849C-5DA79903E56B}"/>
-    <hyperlink ref="E11" r:id="rId10" xr:uid="{7AF80F05-0C06-45C1-91E0-2242269F2FE5}"/>
-    <hyperlink ref="E12" r:id="rId11" xr:uid="{B7CF1F01-045F-4ECC-872D-B2476A6EDE30}"/>
-    <hyperlink ref="E13" r:id="rId12" xr:uid="{5202DE9A-B0BB-433D-AE08-D6B473C43206}"/>
-    <hyperlink ref="E14" r:id="rId13" xr:uid="{7456791F-CCE6-4113-8CF5-F1DD5986DDA2}"/>
-    <hyperlink ref="E15" r:id="rId14" xr:uid="{60F725A1-3EF6-4F33-892A-7B3C9FD981A6}"/>
-    <hyperlink ref="E17" r:id="rId15" xr:uid="{90011979-115E-4DAA-A396-BCE390C1DF51}"/>
+    <hyperlink ref="E2" ns4:id="rId1" ns2:uid="{97722929-2038-4234-80FD-4DEF83C3C193}"/>
+    <hyperlink ref="E3" ns4:id="rId2" ns2:uid="{9D411408-40F9-4801-AE8C-3AEE32AB4F6F}"/>
+    <hyperlink ref="E4" ns4:id="rId3" ns2:uid="{AA8D31E7-236A-4B13-848B-9E3CB9E37B43}"/>
+    <hyperlink ref="E5" ns4:id="rId4" ns2:uid="{55A960DF-E1FD-4872-B20A-AE949F89215A}"/>
+    <hyperlink ref="E6" ns4:id="rId5" ns2:uid="{413665A7-BF97-4CEE-8C6E-ECC7C0E43443}"/>
+    <hyperlink ref="E7" ns4:id="rId6" ns2:uid="{827A3105-6114-485F-A80C-88929EA91C3A}"/>
+    <hyperlink ref="E8" ns4:id="rId7" ns2:uid="{CDB97694-3BF6-4F69-B0C0-E925ADBCD30B}"/>
+    <hyperlink ref="E9" ns4:id="rId8" ns2:uid="{FDF973CA-B570-43F4-9F76-88BAF56A975E}"/>
+    <hyperlink ref="E10" ns4:id="rId9" ns2:uid="{B7BB62B8-3423-4809-849C-5DA79903E56B}"/>
+    <hyperlink ref="E11" ns4:id="rId10" ns2:uid="{7AF80F05-0C06-45C1-91E0-2242269F2FE5}"/>
+    <hyperlink ref="E12" ns4:id="rId11" ns2:uid="{B7CF1F01-045F-4ECC-872D-B2476A6EDE30}"/>
+    <hyperlink ref="E13" ns4:id="rId12" ns2:uid="{5202DE9A-B0BB-433D-AE08-D6B473C43206}"/>
+    <hyperlink ref="E14" ns4:id="rId13" ns2:uid="{7456791F-CCE6-4113-8CF5-F1DD5986DDA2}"/>
+    <hyperlink ref="E15" ns4:id="rId14" ns2:uid="{60F725A1-3EF6-4F33-892A-7B3C9FD981A6}"/>
+    <hyperlink ref="E17" ns4:id="rId15" ns2:uid="{90011979-115E-4DAA-A396-BCE390C1DF51}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId16"/>
+  <pageSetup paperSize="9" orientation="portrait" ns4:id="rId16"/>
 </worksheet>
 </file>
</xml_diff>